<commit_message>
final version for 2026
</commit_message>
<xml_diff>
--- a/bart/validation.xlsx
+++ b/bart/validation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uttam\Desktop\Sports\basketball\bart\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBAAFDCD-2806-4378-BE67-34F89C9E64C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2EDA09D-CCF9-420F-8808-E1A2E839CE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8CF2FCA8-9615-4DD6-B0F6-7A2F5E6CE65C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{8CF2FCA8-9615-4DD6-B0F6-7A2F5E6CE65C}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -197,12 +197,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -217,12 +223,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -560,9 +569,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9E3D10D-0A18-4888-B8BA-67BCEF22A05F}">
   <dimension ref="A1:M13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -601,7 +610,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -609,13 +618,13 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4229</v>
       </c>
       <c r="D2" s="1">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E2" s="1">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F2" s="1">
         <v>10</v>
@@ -627,22 +636,22 @@
         <v>2</v>
       </c>
       <c r="I2" s="1">
-        <v>55.8508</v>
+        <v>58.7806</v>
       </c>
       <c r="J2" s="1">
-        <v>25.445899999999899</v>
+        <v>26.574999999999999</v>
       </c>
       <c r="K2" s="1">
-        <v>10.864699999999999</v>
+        <v>11.6076</v>
       </c>
       <c r="L2" s="1">
-        <v>4.4044999999999996</v>
+        <v>4.1097999999999999</v>
       </c>
       <c r="M2" s="1">
-        <v>0.3513</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.26879999999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -650,10 +659,10 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4294</v>
       </c>
       <c r="D3" s="1">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E3" s="1">
         <v>26</v>
@@ -668,22 +677,22 @@
         <v>1</v>
       </c>
       <c r="I3" s="1">
-        <v>45.441200000000002</v>
+        <v>57.3048</v>
       </c>
       <c r="J3" s="1">
-        <v>20.629899999999999</v>
+        <v>26.968399999999999</v>
       </c>
       <c r="K3" s="1">
-        <v>8.8491999999999909</v>
+        <v>12.4772</v>
       </c>
       <c r="L3" s="1">
-        <v>3.6377999999999999</v>
+        <v>4.5709999999999997</v>
       </c>
       <c r="M3" s="1">
-        <v>0.34510000000000002</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.42759999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -691,13 +700,13 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4199</v>
       </c>
       <c r="D4" s="1">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E4" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" s="1">
         <v>11</v>
@@ -709,22 +718,22 @@
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>48.482900000000001</v>
+        <v>56.692100000000003</v>
       </c>
       <c r="J4" s="1">
-        <v>21.515999999999998</v>
+        <v>25.629000000000001</v>
       </c>
       <c r="K4" s="1">
-        <v>9.0712999999999901</v>
+        <v>11.2638</v>
       </c>
       <c r="L4" s="1">
-        <v>3.6162999999999998</v>
+        <v>4.3452999999999999</v>
       </c>
       <c r="M4" s="1">
-        <v>0.29649999999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.36270000000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -732,10 +741,10 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4257</v>
       </c>
       <c r="D5" s="1">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E5" s="1">
         <v>29</v>
@@ -750,22 +759,22 @@
         <v>1</v>
       </c>
       <c r="I5" s="1">
-        <v>51.6282</v>
+        <v>64.395399999999995</v>
       </c>
       <c r="J5" s="1">
-        <v>22.8245</v>
+        <v>31.0427</v>
       </c>
       <c r="K5" s="1">
-        <v>9.3249999999999993</v>
+        <v>13.1413999999999</v>
       </c>
       <c r="L5" s="1">
-        <v>3.6371000000000002</v>
+        <v>5.4851000000000001</v>
       </c>
       <c r="M5" s="1">
-        <v>0.28149999999999997</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.53110000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -773,7 +782,7 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4235</v>
       </c>
       <c r="D6" s="1">
         <v>60</v>
@@ -791,22 +800,22 @@
         <v>1</v>
       </c>
       <c r="I6" s="1">
-        <v>57.3004999999999</v>
+        <v>62.447600000000001</v>
       </c>
       <c r="J6" s="1">
-        <v>26.193300000000001</v>
+        <v>28.161200000000001</v>
       </c>
       <c r="K6" s="1">
-        <v>10.875299999999999</v>
+        <v>11.340399999999899</v>
       </c>
       <c r="L6" s="1">
-        <v>4.2797000000000001</v>
+        <v>5.1481999999999903</v>
       </c>
       <c r="M6" s="1">
-        <v>0.3322</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.36159999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -814,7 +823,7 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4179</v>
       </c>
       <c r="D7" s="1">
         <v>62</v>
@@ -832,22 +841,22 @@
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>65.423599999999894</v>
+        <v>62.389499999999998</v>
       </c>
       <c r="J7" s="1">
-        <v>30.019500000000001</v>
+        <v>28.176500000000001</v>
       </c>
       <c r="K7" s="1">
-        <v>12.545199999999999</v>
+        <v>11.325299999999899</v>
       </c>
       <c r="L7" s="1">
-        <v>4.9380999999999897</v>
+        <v>4.6325000000000003</v>
       </c>
       <c r="M7" s="1">
-        <v>0.3982</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.62209999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -855,7 +864,7 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4197</v>
       </c>
       <c r="D8" s="1">
         <v>56</v>
@@ -873,22 +882,22 @@
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>58.0870999999999</v>
+        <v>60.985199999999899</v>
       </c>
       <c r="J8" s="1">
-        <v>24.167999999999999</v>
+        <v>26.413399999999999</v>
       </c>
       <c r="K8" s="1">
-        <v>9.3472000000000008</v>
+        <v>9.4261999999999997</v>
       </c>
       <c r="L8" s="1">
-        <v>3.4508000000000001</v>
+        <v>3.7147999999999999</v>
       </c>
       <c r="M8" s="1">
-        <v>0.2485</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.16869999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -896,13 +905,13 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4260</v>
       </c>
       <c r="D9" s="1">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E9" s="1">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F9" s="1">
         <v>8</v>
@@ -914,22 +923,22 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>50.451900000000002</v>
+        <v>60.673999999999999</v>
       </c>
       <c r="J9" s="1">
-        <v>20.535</v>
+        <v>27.030799999999999</v>
       </c>
       <c r="K9" s="1">
-        <v>7.8236999999999997</v>
+        <v>10.5341</v>
       </c>
       <c r="L9" s="1">
-        <v>2.8458999999999999</v>
+        <v>4.024</v>
       </c>
       <c r="M9" s="1">
-        <v>0.1925</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.19470000000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -937,13 +946,13 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>4414</v>
       </c>
       <c r="D10" s="1">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E10" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F10" s="1">
         <v>6</v>
@@ -955,22 +964,22 @@
         <v>0</v>
       </c>
       <c r="I10" s="1">
-        <v>54.310499999999998</v>
+        <v>58.952199999999898</v>
       </c>
       <c r="J10" s="1">
-        <v>23.465199999999999</v>
+        <v>26.161300000000001</v>
       </c>
       <c r="K10" s="1">
-        <v>9.3996999999999993</v>
+        <v>11.105899999999901</v>
       </c>
       <c r="L10" s="1">
-        <v>3.5752000000000002</v>
+        <v>4.2966999999999897</v>
       </c>
       <c r="M10" s="1">
-        <v>0.26439999999999902</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.29430000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -978,7 +987,7 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>4440</v>
       </c>
       <c r="D11" s="1">
         <v>37</v>
@@ -996,22 +1005,22 @@
         <v>1</v>
       </c>
       <c r="I11" s="1">
-        <v>52.577799999999897</v>
+        <v>53.597499999999997</v>
       </c>
       <c r="J11" s="1">
-        <v>23.200700000000001</v>
+        <v>22.969100000000001</v>
       </c>
       <c r="K11" s="1">
-        <v>9.2614000000000001</v>
+        <v>9.5451999999999906</v>
       </c>
       <c r="L11" s="1">
-        <v>3.5086999999999899</v>
+        <v>3.38119999999999</v>
       </c>
       <c r="M11" s="1">
-        <v>0.24249999999999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.23419999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1019,7 +1028,7 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>4412</v>
       </c>
       <c r="D12" s="1">
         <v>28</v>
@@ -1037,22 +1046,22 @@
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>50.265899999999903</v>
+        <v>56.994799999999998</v>
       </c>
       <c r="J12" s="1">
-        <v>20.382199999999902</v>
+        <v>23.056999999999999</v>
       </c>
       <c r="K12" s="1">
-        <v>7.8174000000000001</v>
+        <v>8.2279</v>
       </c>
       <c r="L12" s="1">
-        <v>2.9885000000000002</v>
+        <v>2.7616000000000001</v>
       </c>
       <c r="M12" s="1">
-        <v>0.235599999999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+        <v>0.1469</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1060,7 +1069,7 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>4443</v>
       </c>
       <c r="D13" s="1">
         <v>26</v>
@@ -1078,19 +1087,19 @@
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>57.218299999999999</v>
+        <v>62.497999999999998</v>
       </c>
       <c r="J13" s="1">
-        <v>25.117999999999999</v>
+        <v>27.4633</v>
       </c>
       <c r="K13" s="1">
-        <v>10.159000000000001</v>
+        <v>11.143000000000001</v>
       </c>
       <c r="L13" s="1">
-        <v>3.9390999999999998</v>
+        <v>4.0418999999999903</v>
       </c>
       <c r="M13" s="1">
-        <v>0.30590000000000001</v>
+        <v>0.34699999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -1101,9 +1110,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD7FA1E2-9557-425C-9EE9-5E8EDDD2FE6A}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1118,7 +1127,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1126,16 +1135,16 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4229</v>
       </c>
       <c r="D2" s="1">
-        <v>0.57262845471944901</v>
+        <v>0.63638791025548302</v>
       </c>
       <c r="E2" s="1">
-        <v>0.71381395210041099</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.60138702758571905</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1143,16 +1152,16 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4294</v>
       </c>
       <c r="D3" s="1">
-        <v>0.59369842964575503</v>
+        <v>0.65156536818578303</v>
       </c>
       <c r="E3" s="1">
-        <v>0.66999176791022996</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.58580277877630604</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1160,16 +1169,16 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4199</v>
       </c>
       <c r="D4" s="1">
-        <v>0.55901500762131795</v>
+        <v>0.59197729414143896</v>
       </c>
       <c r="E4" s="1">
-        <v>0.71898230001768104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.64550037920175596</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1177,16 +1186,16 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4257</v>
       </c>
       <c r="D5" s="1">
-        <v>0.59009683099139798</v>
+        <v>0.64566953631094604</v>
       </c>
       <c r="E5" s="1">
-        <v>0.70039937526636398</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.621766035385247</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1194,16 +1203,16 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4235</v>
       </c>
       <c r="D6" s="1">
-        <v>0.60333573314661304</v>
+        <v>0.66355322953615703</v>
       </c>
       <c r="E6" s="1">
-        <v>0.71364316579987896</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.61381830413296201</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1211,16 +1220,16 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4179</v>
       </c>
       <c r="D7" s="1">
-        <v>0.59072167143405896</v>
+        <v>0.628840893093077</v>
       </c>
       <c r="E7" s="1">
-        <v>0.74312921769596296</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.62697867372251304</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1228,16 +1237,16 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4197</v>
       </c>
       <c r="D8" s="1">
-        <v>0.59025162286133803</v>
+        <v>0.63877008211500796</v>
       </c>
       <c r="E8" s="1">
-        <v>0.73630383429213997</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.62641996706551595</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1245,16 +1254,16 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4260</v>
       </c>
       <c r="D9" s="1">
-        <v>0.59114689972465295</v>
+        <v>0.66964831688599902</v>
       </c>
       <c r="E9" s="1">
-        <v>0.71637106079276403</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.61253177295994798</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1262,16 +1271,16 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>4414</v>
       </c>
       <c r="D10" s="1">
-        <v>0.56491579691364402</v>
+        <v>0.63620995110838896</v>
       </c>
       <c r="E10" s="1">
-        <v>0.71467497618206499</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.57893461887341302</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1279,16 +1288,16 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>4440</v>
       </c>
       <c r="D11" s="1">
-        <v>0.55897849677761102</v>
+        <v>0.649814851107958</v>
       </c>
       <c r="E11" s="1">
-        <v>0.70373742526880501</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.54120054702287002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1296,16 +1305,16 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>4412</v>
       </c>
       <c r="D12" s="1">
-        <v>0.48084919936346898</v>
+        <v>0.56931175706499004</v>
       </c>
       <c r="E12" s="1">
-        <v>0.73203595611333605</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+        <v>0.53959117062155704</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1313,13 +1322,13 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>4443</v>
       </c>
       <c r="D13" s="1">
-        <v>0.46710625006842399</v>
+        <v>0.54934102488526704</v>
       </c>
       <c r="E13" s="1">
-        <v>0.74837017265326999</v>
+        <v>0.54980665354188196</v>
       </c>
     </row>
   </sheetData>
@@ -1330,9 +1339,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834031E8-EFDD-445C-BEA4-4000BC5A8F34}">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1356,7 +1365,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1364,25 +1373,25 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" s="1">
-        <v>0.64432877013657797</v>
+        <v>0.60442981155403397</v>
       </c>
       <c r="E2" s="1">
-        <v>0.78254065159730002</v>
+        <v>0.78078528959579996</v>
       </c>
       <c r="F2" s="1">
-        <v>0.710777844271274</v>
+        <v>0.72207366267684203</v>
       </c>
       <c r="G2" s="1">
-        <v>0.48492270581866198</v>
+        <v>0.49462349966121899</v>
       </c>
       <c r="H2" s="1">
-        <v>0.205556612948259</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.21004201260420099</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1390,25 +1399,25 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D3" s="1">
-        <v>0.436188441236044</v>
+        <v>0.488031133130093</v>
       </c>
       <c r="E3" s="1">
-        <v>0.86231649850257597</v>
+        <v>0.86469203054747001</v>
       </c>
       <c r="F3" s="1">
-        <v>0.74535599249993001</v>
+        <v>0.75498344352707403</v>
       </c>
       <c r="G3" s="1">
-        <v>0.54889165714378496</v>
+        <v>0.55815630565143803</v>
       </c>
       <c r="H3" s="1">
-        <v>0.40032038451271701</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.407619732292054</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1416,25 +1425,25 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D4" s="1">
-        <v>0.33701812972932499</v>
+        <v>0.22193837432533001</v>
       </c>
       <c r="E4" s="1">
-        <v>0.79793288796170803</v>
+        <v>0.804153333762198</v>
       </c>
       <c r="F4" s="1">
-        <v>0.72015176225511202</v>
+        <v>0.72738405872799405</v>
       </c>
       <c r="G4" s="1">
-        <v>0.544383562614839</v>
+        <v>0.55112199757907798</v>
       </c>
       <c r="H4" s="1">
-        <v>0.28466497871377799</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.28858673308160998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1442,25 +1451,25 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1">
-        <v>0.573899445525338</v>
+        <v>0.56864261843376895</v>
       </c>
       <c r="E5" s="1">
-        <v>0.76452257881580099</v>
+        <v>0.75909124102120995</v>
       </c>
       <c r="F5" s="1">
-        <v>0.64863834863279002</v>
+        <v>0.65495298658311796</v>
       </c>
       <c r="G5" s="1">
-        <v>0.48135986234123201</v>
+        <v>0.48671371862979002</v>
       </c>
       <c r="H5" s="1">
-        <v>0.370986067151996</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.37530475421527099</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1471,7 +1480,7 @@
         <v>86</v>
       </c>
       <c r="D6" s="1">
-        <v>0.57336541246929096</v>
+        <v>0.63563975322186606</v>
       </c>
       <c r="E6" s="1">
         <v>0.77694987973398899</v>
@@ -1486,7 +1495,7 @@
         <v>0.31782730968713402</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1494,23 +1503,21 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1">
-        <v>0.41282836079190599</v>
+        <v>0.38284083544956898</v>
       </c>
       <c r="E7" s="1">
-        <v>0.80638606037969895</v>
+        <v>0.790617088196229</v>
       </c>
       <c r="F7" s="1">
-        <v>0.57004432835591101</v>
-      </c>
-      <c r="G7" s="1">
-        <v>1.79461500985255E-3</v>
-      </c>
+        <v>0.547311688975891</v>
+      </c>
+      <c r="G7" s="3"/>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1518,25 +1525,25 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D8" s="1">
-        <v>0.36889341552695398</v>
+        <v>0.35613841564991799</v>
       </c>
       <c r="E8" s="1">
-        <v>0.81384130046198899</v>
+        <v>0.81928803037291398</v>
       </c>
       <c r="F8" s="1">
-        <v>0.65226876780553</v>
+        <v>0.65918172604009995</v>
       </c>
       <c r="G8" s="1">
-        <v>0.50090826596203297</v>
+        <v>0.50693816326043395</v>
       </c>
       <c r="H8" s="1">
-        <v>0.33729250475845701</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.34163186146365598</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1544,25 +1551,25 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D9" s="1">
-        <v>0.52437527773238402</v>
+        <v>0.52419422279504302</v>
       </c>
       <c r="E9" s="1">
-        <v>0.84780829697410398</v>
+        <v>0.85083079603306599</v>
       </c>
       <c r="F9" s="1">
-        <v>0.66947450639184303</v>
+        <v>0.67512747051891997</v>
       </c>
       <c r="G9" s="1">
-        <v>0.42553769653796603</v>
+        <v>0.42986347681054698</v>
       </c>
       <c r="H9" s="1">
-        <v>0.306044563332868</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.30927685641354302</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1573,7 +1580,7 @@
         <v>77</v>
       </c>
       <c r="D10" s="1">
-        <v>0.33443092717825701</v>
+        <v>0.34801985296318499</v>
       </c>
       <c r="E10" s="1">
         <v>0.79280672936186503</v>
@@ -1588,7 +1595,7 @@
         <v>0.27551938438899098</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1596,25 +1603,25 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D11" s="1">
-        <v>0.480519937308237</v>
+        <v>0.475890819682942</v>
       </c>
       <c r="E11" s="1">
-        <v>0.75005860061734897</v>
+        <v>0.75319830875254301</v>
       </c>
       <c r="F11" s="1">
-        <v>0.57286671883027496</v>
+        <v>0.57596073584122798</v>
       </c>
       <c r="G11" s="1">
-        <v>0.32908687544372001</v>
+        <v>0.331082141794728</v>
       </c>
       <c r="H11" s="1">
-        <v>0.19245008972987501</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.19364916731036999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1625,7 +1632,7 @@
         <v>81</v>
       </c>
       <c r="D12" s="1">
-        <v>0.50199869025200605</v>
+        <v>0.45702412670307202</v>
       </c>
       <c r="E12" s="1">
         <v>0.78106400224933903</v>
@@ -1638,7 +1645,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1646,19 +1653,19 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13" s="1">
-        <v>0.60712244176604102</v>
+        <v>0.539416398798093</v>
       </c>
       <c r="E13" s="1">
-        <v>0.79814985395523896</v>
+        <v>0.80077920946439296</v>
       </c>
       <c r="F13" s="1">
-        <v>0.60314788851100298</v>
+        <v>0.60613447995959502</v>
       </c>
       <c r="G13" s="1">
-        <v>0.31962394847466902</v>
+        <v>0.32145135081780801</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -1673,9 +1680,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0481036-F6AB-449C-BC56-993E67FE8301}">
   <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1699,7 +1706,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1707,25 +1714,25 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" s="1">
-        <v>0.46424895393115401</v>
+        <v>0.42850683119785099</v>
       </c>
       <c r="E2" s="1">
-        <v>0.64348945208778596</v>
+        <v>0.64224842494840795</v>
       </c>
       <c r="F2" s="1">
-        <v>0.58447832024147595</v>
+        <v>0.59395416221405295</v>
       </c>
       <c r="G2" s="1">
-        <v>0.39875582902338103</v>
+        <v>0.40686110231961498</v>
       </c>
       <c r="H2" s="1">
-        <v>0.169030850945703</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.172773685116272</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1733,25 +1740,25 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D3" s="1">
-        <v>0.29255900293866</v>
+        <v>0.32888550162948299</v>
       </c>
       <c r="E3" s="1">
-        <v>0.71068968321943604</v>
+        <v>0.71290623094320504</v>
       </c>
       <c r="F3" s="1">
-        <v>0.61429511683395099</v>
+        <v>0.62245560515763398</v>
       </c>
       <c r="G3" s="1">
-        <v>0.45237640543200502</v>
+        <v>0.46017899330842199</v>
       </c>
       <c r="H3" s="1">
-        <v>0.32992940266093701</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.33606722016672202</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1759,25 +1766,25 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D4" s="1">
-        <v>0.244858212561824</v>
+        <v>0.153431635788181</v>
       </c>
       <c r="E4" s="1">
-        <v>0.65601824471746994</v>
+        <v>0.66126173391883303</v>
       </c>
       <c r="F4" s="1">
-        <v>0.59207071438251402</v>
+        <v>0.59813374353507198</v>
       </c>
       <c r="G4" s="1">
-        <v>0.44756339109156701</v>
+        <v>0.45319203741275799</v>
       </c>
       <c r="H4" s="1">
-        <v>0.23403649916646899</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.237307184452895</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1785,25 +1792,25 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1">
-        <v>0.40582278280961198</v>
+        <v>0.390854546480221</v>
       </c>
       <c r="E5" s="1">
-        <v>0.62797923491370999</v>
+        <v>0.62360956446232296</v>
       </c>
       <c r="F5" s="1">
-        <v>0.53279186932718603</v>
+        <v>0.53805777834681101</v>
       </c>
       <c r="G5" s="1">
-        <v>0.39538923564485901</v>
+        <v>0.39984564923214599</v>
       </c>
       <c r="H5" s="1">
-        <v>0.30472814416366301</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.308320820566924</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1814,7 +1821,7 @@
         <v>86</v>
       </c>
       <c r="D6" s="1">
-        <v>0.40597209313837601</v>
+        <v>0.44417078839044999</v>
       </c>
       <c r="E6" s="1">
         <v>0.63805449852787199</v>
@@ -1829,7 +1836,7 @@
         <v>0.26100930058746902</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1837,23 +1844,21 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1">
-        <v>0.291886610846676</v>
+        <v>0.26474306970890998</v>
       </c>
       <c r="E7" s="1">
-        <v>0.66176217730659703</v>
+        <v>0.64896076832351102</v>
       </c>
       <c r="F7" s="1">
-        <v>0.46780790793488902</v>
-      </c>
-      <c r="G7" s="1">
-        <v>1.4727540500736301E-3</v>
-      </c>
+        <v>0.44924884560814998</v>
+      </c>
+      <c r="G7" s="1"/>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1861,25 +1866,25 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D8" s="1">
-        <v>0.252413585988912</v>
+        <v>0.236100961376361</v>
       </c>
       <c r="E8" s="1">
-        <v>0.66885605405993798</v>
+        <v>0.67345061252353899</v>
       </c>
       <c r="F8" s="1">
-        <v>0.536067552695209</v>
+        <v>0.54184404105594897</v>
       </c>
       <c r="G8" s="1">
-        <v>0.41167181614791898</v>
+        <v>0.416700603332266</v>
       </c>
       <c r="H8" s="1">
-        <v>0.27720408594239299</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.28081966027934602</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1887,25 +1892,25 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D9" s="1">
-        <v>0.38465154889666298</v>
+        <v>0.37092248826718299</v>
       </c>
       <c r="E9" s="1">
-        <v>0.69594430518779904</v>
+        <v>0.69850704213492898</v>
       </c>
       <c r="F9" s="1">
-        <v>0.54955462438231795</v>
+        <v>0.55425978313775104</v>
       </c>
       <c r="G9" s="1">
-        <v>0.34931309071321398</v>
+        <v>0.35290526284276902</v>
       </c>
       <c r="H9" s="1">
-        <v>0.25122421158813202</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.25390719656769101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1916,7 +1921,7 @@
         <v>77</v>
       </c>
       <c r="D10" s="1">
-        <v>0.22594428632852101</v>
+        <v>0.239123674901037</v>
       </c>
       <c r="E10" s="1">
         <v>0.65151382684907699</v>
@@ -1931,7 +1936,7 @@
         <v>0.22641670642586301</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1939,25 +1944,25 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D11" s="1">
-        <v>0.33122235901430902</v>
+        <v>0.331330302528836</v>
       </c>
       <c r="E11" s="1">
-        <v>0.61623602251331999</v>
+        <v>0.61886390659923696</v>
       </c>
       <c r="F11" s="1">
-        <v>0.47065803652096699</v>
+        <v>0.47323700397152502</v>
       </c>
       <c r="G11" s="1">
-        <v>0.27037245758912798</v>
+        <v>0.27203298957969901</v>
       </c>
       <c r="H11" s="1">
-        <v>0.158113883008418</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.15911145683514599</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1968,7 +1973,7 @@
         <v>81</v>
       </c>
       <c r="D12" s="1">
-        <v>0.35392224169409497</v>
+        <v>0.31803461450809101</v>
       </c>
       <c r="E12" s="1">
         <v>0.64166065413248397</v>
@@ -1981,7 +1986,7 @@
       </c>
       <c r="H12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1989,19 +1994,19 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D13" s="1">
-        <v>0.441361955763799</v>
+        <v>0.383919791883987</v>
       </c>
       <c r="E13" s="1">
-        <v>0.65550886855228696</v>
+        <v>0.65771383810017003</v>
       </c>
       <c r="F13" s="1">
-        <v>0.49535659000411397</v>
+        <v>0.49784388818701297</v>
       </c>
       <c r="G13" s="1">
-        <v>0.26250250098848599</v>
+        <v>0.26402159198198499</v>
       </c>
       <c r="H13" s="1"/>
     </row>
@@ -2013,9 +2018,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3208696C-FD95-4C0F-8D26-9B4D6AE84141}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2036,7 +2041,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2044,22 +2049,22 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4229</v>
       </c>
       <c r="D2" s="1">
-        <v>8.8783498963625196E-3</v>
+        <v>9.1408558477181299E-3</v>
       </c>
       <c r="E2" s="1">
-        <v>5.1238380918512396E-3</v>
+        <v>5.5044721920075599E-3</v>
       </c>
       <c r="F2" s="1">
-        <v>1.59728175370859E-3</v>
+        <v>1.9306085599432401E-3</v>
       </c>
       <c r="G2" s="1">
-        <v>3.9246256248729898E-4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>4.52804861669425E-4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2067,22 +2072,22 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4294</v>
       </c>
       <c r="D3" s="1">
-        <v>8.78056051455923E-3</v>
+        <v>9.5878218118304603E-3</v>
       </c>
       <c r="E3" s="1">
-        <v>4.1848717969684797E-3</v>
+        <v>4.9176623847228696E-3</v>
       </c>
       <c r="F3" s="1">
-        <v>1.66575752692461E-3</v>
+        <v>1.8858828039124301E-3</v>
       </c>
       <c r="G3" s="1">
-        <v>5.6077966094934199E-4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>5.9301030274801995E-4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2090,22 +2095,22 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4199</v>
       </c>
       <c r="D4" s="1">
-        <v>9.8938184530958703E-3</v>
+        <v>1.01175779352226E-2</v>
       </c>
       <c r="E4" s="1">
-        <v>5.0721005342721E-3</v>
+        <v>5.5454200285782297E-3</v>
       </c>
       <c r="F4" s="1">
-        <v>1.91321255539449E-3</v>
+        <v>2.2164986472969698E-3</v>
       </c>
       <c r="G4" s="1">
-        <v>8.4019271277697202E-4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>9.3140748035246395E-4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2113,22 +2118,22 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4257</v>
       </c>
       <c r="D5" s="1">
-        <v>9.1312717792155201E-3</v>
+        <v>1.00340743904157E-2</v>
       </c>
       <c r="E5" s="1">
-        <v>4.8025344177112803E-3</v>
+        <v>5.3087964176650199E-3</v>
       </c>
       <c r="F5" s="1">
-        <v>2.1900323291548702E-3</v>
+        <v>2.3873036739487899E-3</v>
       </c>
       <c r="G5" s="1">
-        <v>1.11152014355034E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1.1226275428705601E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2136,22 +2141,22 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4235</v>
       </c>
       <c r="D6" s="1">
-        <v>1.0121301406028699E-2</v>
+        <v>1.08118425312868E-2</v>
       </c>
       <c r="E6" s="1">
-        <v>3.87079550273113E-3</v>
+        <v>4.4020146587957498E-3</v>
       </c>
       <c r="F6" s="1">
-        <v>1.26603937891968E-3</v>
+        <v>1.48822212987013E-3</v>
       </c>
       <c r="G6" s="1">
-        <v>5.29679670240744E-4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>5.6037157969303396E-4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2159,22 +2164,22 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4179</v>
       </c>
       <c r="D7" s="1">
-        <v>1.0987743536459401E-2</v>
+        <v>1.13648117755443E-2</v>
       </c>
       <c r="E7" s="1">
-        <v>4.6830852199958601E-3</v>
+        <v>5.1217343598947097E-3</v>
       </c>
       <c r="F7" s="1">
-        <v>1.09941110927494E-3</v>
+        <v>1.0145546661880799E-3</v>
       </c>
       <c r="G7" s="1">
-        <v>3.0841810576327197E-4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>3.1903029672170302E-4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2182,22 +2187,22 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4197</v>
       </c>
       <c r="D8" s="1">
-        <v>9.6159061853759008E-3</v>
+        <v>1.0596670326423601E-2</v>
       </c>
       <c r="E8" s="1">
-        <v>4.5395590978372802E-3</v>
+        <v>5.1991840743388102E-3</v>
       </c>
       <c r="F8" s="1">
-        <v>1.40399819155509E-3</v>
+        <v>1.66424915415773E-3</v>
       </c>
       <c r="G8" s="1">
-        <v>5.7541684860967996E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>6.5124546580891103E-4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2205,22 +2210,22 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4260</v>
       </c>
       <c r="D9" s="1">
-        <v>8.7352198928084199E-3</v>
+        <v>9.5928781877934206E-3</v>
       </c>
       <c r="E9" s="1">
-        <v>4.5705718339504901E-3</v>
+        <v>5.1436836854460103E-3</v>
       </c>
       <c r="F9" s="1">
-        <v>1.09998344767101E-3</v>
+        <v>1.29354511971831E-3</v>
       </c>
       <c r="G9" s="1">
-        <v>4.7964939972714799E-4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>5.7172436619718197E-4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2228,22 +2233,22 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>4414</v>
       </c>
       <c r="D10" s="1">
-        <v>7.3407844121661098E-3</v>
+        <v>7.7488222972360602E-3</v>
       </c>
       <c r="E10" s="1">
-        <v>3.7558332696431998E-3</v>
+        <v>3.9680949456275399E-3</v>
       </c>
       <c r="F10" s="1">
-        <v>1.08081573211152E-3</v>
+        <v>1.2209298119619299E-3</v>
       </c>
       <c r="G10" s="1">
-        <v>3.27676166894131E-4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>3.8815271635704498E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2251,22 +2256,22 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>4440</v>
       </c>
       <c r="D11" s="1">
-        <v>6.0152762875411697E-3</v>
+        <v>6.2864659256756704E-3</v>
       </c>
       <c r="E11" s="1">
-        <v>2.52500853904282E-3</v>
+        <v>2.8904040563063E-3</v>
       </c>
       <c r="F11" s="1">
-        <v>5.4414315055221802E-4</v>
+        <v>6.6649431531531499E-4</v>
       </c>
       <c r="G11" s="1">
-        <v>1.28151464832396E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1.29516441441441E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2274,22 +2279,22 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>4412</v>
       </c>
       <c r="D12" s="1">
-        <v>5.0320439847715698E-3</v>
+        <v>5.8038057026291896E-3</v>
       </c>
       <c r="E12" s="1">
-        <v>1.7236147051932799E-3</v>
+        <v>2.0900905983680801E-3</v>
       </c>
       <c r="F12" s="1">
-        <v>5.2869731354939398E-4</v>
+        <v>6.3537638485947404E-4</v>
       </c>
       <c r="G12" s="2">
-        <v>3.3648135493947598E-5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+        <v>2.1190457842248399E-5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2297,19 +2302,19 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>4443</v>
       </c>
       <c r="D13" s="1">
-        <v>3.77344320883848E-3</v>
+        <v>4.3202351159126696E-3</v>
       </c>
       <c r="E13" s="1">
-        <v>1.3744470238560801E-3</v>
+        <v>1.70903741841098E-3</v>
       </c>
       <c r="F13" s="1">
-        <v>4.20913640985529E-4</v>
+        <v>5.1590753094755797E-4</v>
       </c>
       <c r="G13" s="2">
-        <v>7.1236173249902197E-5</v>
+        <v>8.4144836821967094E-5</v>
       </c>
     </row>
   </sheetData>
@@ -2320,9 +2325,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26959CBB-4390-4525-A282-958F0D73204D}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2343,7 +2348,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2351,22 +2356,22 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4229</v>
       </c>
       <c r="D2" s="1">
-        <v>4.9715254814285598E-2</v>
+        <v>3.5226449547426798E-2</v>
       </c>
       <c r="E2" s="1">
-        <v>3.33357742591852E-2</v>
+        <v>2.1374294856302101E-2</v>
       </c>
       <c r="F2" s="1">
-        <v>1.30105635285361E-2</v>
+        <v>8.5466502200205706E-3</v>
       </c>
       <c r="G2" s="1">
-        <v>1.8359155628506899E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>2.1073720444192302E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2374,22 +2379,22 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4294</v>
       </c>
       <c r="D3" s="1">
-        <v>5.5386656054931503E-2</v>
+        <v>3.7312863115091903E-2</v>
       </c>
       <c r="E3" s="1">
-        <v>2.3750341739311599E-2</v>
+        <v>2.61032198234563E-2</v>
       </c>
       <c r="F3" s="1">
-        <v>1.27167538023139E-2</v>
+        <v>7.5647965754941397E-3</v>
       </c>
       <c r="G3" s="1">
-        <v>2.3091143856933901E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>2.6239783101289801E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2397,22 +2402,22 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4199</v>
       </c>
       <c r="D4" s="1">
-        <v>6.0786695474619998E-2</v>
+        <v>4.1942243020467201E-2</v>
       </c>
       <c r="E4" s="1">
-        <v>4.7380959000200201E-2</v>
+        <v>2.47630532287073E-2</v>
       </c>
       <c r="F4" s="1">
-        <v>8.76949555018669E-3</v>
+        <v>9.2588189627094992E-3</v>
       </c>
       <c r="G4" s="1">
-        <v>4.6051012535165397E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>4.6930270650224802E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2420,22 +2425,22 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4257</v>
       </c>
       <c r="D5" s="1">
-        <v>4.8996082457169597E-2</v>
+        <v>4.49787401299458E-2</v>
       </c>
       <c r="E5" s="1">
-        <v>2.7736026322010901E-2</v>
+        <v>2.2390653217525001E-2</v>
       </c>
       <c r="F5" s="1">
-        <v>9.5877420000581807E-3</v>
+        <v>1.0668891993295E-2</v>
       </c>
       <c r="G5" s="1">
-        <v>4.5129289845963899E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>4.5324245602510402E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2443,22 +2448,22 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4235</v>
       </c>
       <c r="D6" s="1">
-        <v>4.8793954146253399E-2</v>
+        <v>4.3364102628502203E-2</v>
       </c>
       <c r="E6" s="1">
-        <v>2.3665252131973302E-2</v>
+        <v>1.9213637524045001E-2</v>
       </c>
       <c r="F6" s="1">
-        <v>6.3068590874193796E-3</v>
+        <v>7.3058482166365197E-3</v>
       </c>
       <c r="G6" s="1">
-        <v>2.41777490178366E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>2.9133719783417901E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2466,22 +2471,22 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4179</v>
       </c>
       <c r="D7" s="1">
-        <v>6.7927460764939607E-2</v>
+        <v>4.3580714981342798E-2</v>
       </c>
       <c r="E7" s="1">
-        <v>2.61303848573009E-2</v>
+        <v>2.2813743790332301E-2</v>
       </c>
       <c r="F7" s="1">
-        <v>5.7855324728471403E-3</v>
+        <v>6.21241758171293E-3</v>
       </c>
       <c r="G7" s="1">
-        <v>2.3975376012372899E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>2.5966597889832098E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2489,22 +2494,22 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4197</v>
       </c>
       <c r="D8" s="1">
-        <v>4.3146216897040901E-2</v>
+        <v>4.0053968848260298E-2</v>
       </c>
       <c r="E8" s="1">
-        <v>2.5162613330814501E-2</v>
+        <v>2.2869828368970401E-2</v>
       </c>
       <c r="F8" s="1">
-        <v>6.3477566688662796E-3</v>
+        <v>7.1987154380427501E-3</v>
       </c>
       <c r="G8" s="1">
-        <v>2.45734332225531E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>2.77545762404876E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2512,22 +2517,22 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4260</v>
       </c>
       <c r="D9" s="1">
-        <v>5.7905170064019698E-2</v>
+        <v>4.3445362239783299E-2</v>
       </c>
       <c r="E9" s="1">
-        <v>3.8513011257481501E-2</v>
+        <v>2.8855181461940101E-2</v>
       </c>
       <c r="F9" s="1">
-        <v>5.0596162718961604E-3</v>
+        <v>6.1524020478544803E-3</v>
       </c>
       <c r="G9" s="1">
-        <v>1.7198690047920801E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>2.2588610304193298E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2535,22 +2540,22 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>4414</v>
       </c>
       <c r="D10" s="1">
-        <v>4.1481101077679702E-2</v>
+        <v>3.17551221152668E-2</v>
       </c>
       <c r="E10" s="1">
-        <v>2.7836220759408298E-2</v>
+        <v>1.7274185476789699E-2</v>
       </c>
       <c r="F10" s="1">
-        <v>5.0299233281463698E-3</v>
+        <v>5.6884498719626002E-3</v>
       </c>
       <c r="G10" s="1">
-        <v>1.45964132611186E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>1.7924570543712099E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2558,22 +2563,22 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>4440</v>
       </c>
       <c r="D11" s="1">
-        <v>3.0554356909258999E-2</v>
+        <v>2.5017524079890399E-2</v>
       </c>
       <c r="E11" s="1">
-        <v>1.65391508866429E-2</v>
+        <v>1.23409490934317E-2</v>
       </c>
       <c r="F11" s="1">
-        <v>2.5346191648455301E-3</v>
+        <v>3.2858712735872801E-3</v>
       </c>
       <c r="G11" s="1">
-        <v>8.5615411174013605E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>9.4152338556371701E-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2581,22 +2586,22 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>4412</v>
       </c>
       <c r="D12" s="1">
-        <v>2.11124203718756E-2</v>
+        <v>2.43437257239098E-2</v>
       </c>
       <c r="E12" s="1">
-        <v>8.0262190676736404E-3</v>
+        <v>1.0135880909472501E-2</v>
       </c>
       <c r="F12" s="1">
-        <v>2.4525443207471498E-3</v>
+        <v>3.2965378027028898E-3</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2604,16 +2609,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>4443</v>
       </c>
       <c r="D13" s="1">
-        <v>1.6267060767428999E-2</v>
+        <v>1.81624733584188E-2</v>
       </c>
       <c r="E13" s="1">
-        <v>6.3790239037187597E-3</v>
+        <v>8.3212026380079206E-3</v>
       </c>
       <c r="F13" s="1">
-        <v>2.3752838176087101E-3</v>
+        <v>3.0757587531145998E-3</v>
       </c>
       <c r="G13" s="1">
         <v>0</v>
@@ -2627,9 +2632,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88E95CE6-CD40-4D98-91F1-85007EDA77BB}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2650,7 +2655,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2658,22 +2663,22 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4229</v>
       </c>
       <c r="D2" s="1">
-        <v>0.94480020394341302</v>
+        <v>0.96740851918012505</v>
       </c>
       <c r="E2" s="1">
-        <v>0.94732115463284905</v>
+        <v>0.98024404862530501</v>
       </c>
       <c r="F2" s="1">
-        <v>0.93901445734066302</v>
+        <v>0.982033657264754</v>
       </c>
       <c r="G2" s="1">
-        <v>0.99766212644846497</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.99846226638277702</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2681,22 +2686,22 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4294</v>
       </c>
       <c r="D3" s="1">
-        <v>0.94933445172341702</v>
+        <v>0.96201038225578095</v>
       </c>
       <c r="E3" s="1">
-        <v>0.95990762445253197</v>
+        <v>0.95577103309061995</v>
       </c>
       <c r="F3" s="1">
-        <v>0.93392163392163297</v>
+        <v>0.99255801892908002</v>
       </c>
       <c r="G3" s="1">
-        <v>0.99733918712166503</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.99665967528936505</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -2704,22 +2709,22 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4199</v>
       </c>
       <c r="D4" s="1">
-        <v>0.93189254569785696</v>
+        <v>0.94839536174899197</v>
       </c>
       <c r="E4" s="1">
-        <v>0.90235632183907999</v>
+        <v>0.950478645066274</v>
       </c>
       <c r="F4" s="1">
-        <v>0.98265972300841498</v>
+        <v>0.98849526786489506</v>
       </c>
       <c r="G4" s="1">
-        <v>0.980984455958549</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.98581644815256197</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -2727,22 +2732,22 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4257</v>
       </c>
       <c r="D5" s="1">
-        <v>0.95153556821501595</v>
+        <v>0.95623728960235299</v>
       </c>
       <c r="E5" s="1">
-        <v>0.95480844080705196</v>
+        <v>0.96780902358659804</v>
       </c>
       <c r="F5" s="1">
-        <v>0.98508647480070199</v>
+        <v>0.97995681193561002</v>
       </c>
       <c r="G5" s="1">
-        <v>0.99441632928474999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.99560887634282103</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -2750,22 +2755,22 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4235</v>
       </c>
       <c r="D6" s="1">
-        <v>0.95145743736773802</v>
+        <v>0.953874251497006</v>
       </c>
       <c r="E6" s="1">
-        <v>0.95155688825642004</v>
+        <v>0.96888110504234903</v>
       </c>
       <c r="F6" s="1">
-        <v>0.98337132725430598</v>
+        <v>0.98213863259995204</v>
       </c>
       <c r="G6" s="1">
-        <v>0.994871794871794</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.99082388153749201</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -2773,22 +2778,22 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4179</v>
       </c>
       <c r="D7" s="1">
-        <v>0.94960985224334904</v>
+        <v>0.95980866117671004</v>
       </c>
       <c r="E7" s="1">
-        <v>0.95407780174135304</v>
+        <v>0.95929263368463902</v>
       </c>
       <c r="F7" s="1">
-        <v>0.96785861926415795</v>
+        <v>0.95286558109833897</v>
       </c>
       <c r="G7" s="1">
-        <v>0.959710743801652</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.94877932024892198</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -2796,22 +2801,22 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4197</v>
       </c>
       <c r="D8" s="1">
-        <v>0.95998794391688702</v>
+        <v>0.96315158519336197</v>
       </c>
       <c r="E8" s="1">
-        <v>0.95460869565217399</v>
+        <v>0.95871524448705603</v>
       </c>
       <c r="F8" s="1">
-        <v>0.98577728491850602</v>
+        <v>0.98769097636667402</v>
       </c>
       <c r="G8" s="1">
-        <v>0.997045891728496</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.99833094897472496</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -2819,22 +2824,22 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4260</v>
       </c>
       <c r="D9" s="1">
-        <v>0.93768816144087297</v>
+        <v>0.95882092271332198</v>
       </c>
       <c r="E9" s="1">
-        <v>0.91852079644223295</v>
+        <v>0.94919237780178201</v>
       </c>
       <c r="F9" s="1">
-        <v>0.98920310365020503</v>
+        <v>0.98721190028221995</v>
       </c>
       <c r="G9" s="1">
-        <v>0.99980499219968799</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.99953018557669704</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -2842,22 +2847,22 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>4414</v>
       </c>
       <c r="D10" s="1">
-        <v>0.94113847622791902</v>
+        <v>0.95403055334006304</v>
       </c>
       <c r="E10" s="1">
-        <v>0.92966872563504599</v>
+        <v>0.96869478499344197</v>
       </c>
       <c r="F10" s="1">
-        <v>0.98799531524497297</v>
+        <v>0.98916742286751302</v>
       </c>
       <c r="G10" s="1">
-        <v>0.99912229373902794</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.99898005439709803</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -2865,22 +2870,22 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>4440</v>
       </c>
       <c r="D11" s="1">
-        <v>0.96021372660716897</v>
+        <v>0.97652706078779195</v>
       </c>
       <c r="E11" s="1">
-        <v>0.95243561710398394</v>
+        <v>0.98291986889692595</v>
       </c>
       <c r="F11" s="1">
-        <v>0.99932131083963505</v>
+        <v>0.99870378719567099</v>
       </c>
       <c r="G11" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -2888,20 +2893,20 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>4412</v>
       </c>
       <c r="D12" s="1">
-        <v>0.97001374165685095</v>
+        <v>0.96898624869655803</v>
       </c>
       <c r="E12" s="1">
-        <v>0.98386723822059297</v>
+        <v>0.97807316518972898</v>
       </c>
       <c r="F12" s="1">
-        <v>0.99876277918864298</v>
+        <v>0.99758070613139704</v>
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -2909,16 +2914,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>4443</v>
       </c>
       <c r="D13" s="1">
-        <v>0.98686955732946302</v>
+        <v>0.99198899357377901</v>
       </c>
       <c r="E13" s="1">
-        <v>0.99617796942375503</v>
+        <v>0.99568381855111698</v>
       </c>
       <c r="F13" s="1">
-        <v>0.99967390595447703</v>
+        <v>0.99984984984984904</v>
       </c>
       <c r="G13" s="1"/>
     </row>
@@ -2930,9 +2935,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7C1D4F9-388A-41D2-B1F5-AEE3CC4FABF1}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -2953,7 +2958,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -2961,22 +2966,22 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4229</v>
       </c>
       <c r="D2" s="1">
-        <v>0.35115021469762903</v>
+        <v>0.42593409131548898</v>
       </c>
       <c r="E2" s="1">
-        <v>0.36929093762295401</v>
+        <v>0.43248487798135798</v>
       </c>
       <c r="F2" s="1">
-        <v>0.45512485144891002</v>
+        <v>0.34078648486811702</v>
       </c>
       <c r="G2" s="1">
-        <v>0.170454545454545</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.18333333333333299</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -2984,22 +2989,22 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4294</v>
       </c>
       <c r="D3" s="1">
-        <v>0.37069888970507697</v>
+        <v>0.39848067440610502</v>
       </c>
       <c r="E3" s="1">
-        <v>0.33366596199263698</v>
+        <v>0.31052463738351899</v>
       </c>
       <c r="F3" s="1">
-        <v>0.16626336590930799</v>
+        <v>0.18976514225275901</v>
       </c>
       <c r="G3" s="1">
-        <v>0.16254901960784299</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.35658914728682101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -3007,22 +3012,22 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4199</v>
       </c>
       <c r="D4" s="1">
-        <v>0.31110876849887598</v>
+        <v>0.35112855562068401</v>
       </c>
       <c r="E4" s="1">
-        <v>0.26972587264500603</v>
+        <v>0.30285096010917001</v>
       </c>
       <c r="F4" s="1">
-        <v>0.292184595865561</v>
+        <v>0.41389047814340002</v>
       </c>
       <c r="G4" s="1">
-        <v>6.4644470640920895E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>9.0631469979295998E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -3030,22 +3035,22 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4257</v>
       </c>
       <c r="D5" s="1">
-        <v>0.35096739615467398</v>
+        <v>0.37553068439598197</v>
       </c>
       <c r="E5" s="1">
-        <v>0.33219388558840401</v>
+        <v>0.38996561000108598</v>
       </c>
       <c r="F5" s="1">
-        <v>0.19058836903742599</v>
+        <v>0.35243787045077102</v>
       </c>
       <c r="G5" s="1">
-        <v>0.19704202131738299</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.53899944720840198</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -3053,22 +3058,22 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4235</v>
       </c>
       <c r="D6" s="1">
-        <v>0.343879574762885</v>
+        <v>0.38742768451444498</v>
       </c>
       <c r="E6" s="1">
-        <v>0.38815327449100001</v>
+        <v>0.38221020814663498</v>
       </c>
       <c r="F6" s="1">
-        <v>0.48578500676543002</v>
+        <v>0.41155660131931299</v>
       </c>
       <c r="G6" s="1">
-        <v>0.26388888888888801</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.50840336134453701</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -3076,22 +3081,22 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4179</v>
       </c>
       <c r="D7" s="1">
-        <v>0.32449346487441999</v>
+        <v>0.39773989828011402</v>
       </c>
       <c r="E7" s="1">
-        <v>0.28079795006231201</v>
+        <v>0.31724864862357199</v>
       </c>
       <c r="F7" s="1">
-        <v>1.21271799311078E-2</v>
+        <v>9.67774861475648E-3</v>
       </c>
       <c r="G7" s="1">
-        <v>5.0761421319796898E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>4.60829493087557E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -3099,22 +3104,22 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4197</v>
       </c>
       <c r="D8" s="1">
-        <v>0.31021834372271101</v>
+        <v>0.33824026815083702</v>
       </c>
       <c r="E8" s="1">
-        <v>0.23654356239659999</v>
+        <v>0.284849527966128</v>
       </c>
       <c r="F8" s="1">
-        <v>0.26458880009541902</v>
+        <v>0.27381510629130001</v>
       </c>
       <c r="G8" s="1">
-        <v>0.165865384615384</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.22727272727272699</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -3122,22 +3127,22 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4260</v>
       </c>
       <c r="D9" s="1">
-        <v>0.39822902470691302</v>
+        <v>0.468901445377996</v>
       </c>
       <c r="E9" s="1">
-        <v>0.33086844204175297</v>
+        <v>0.40545774500793103</v>
       </c>
       <c r="F9" s="1">
-        <v>0.60428902258511197</v>
+        <v>0.68521305155221801</v>
       </c>
       <c r="G9" s="1">
-        <v>0.63888888888888795</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -3145,22 +3150,22 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>4414</v>
       </c>
       <c r="D10" s="1">
-        <v>0.304555560776958</v>
+        <v>0.349900304094246</v>
       </c>
       <c r="E10" s="1">
-        <v>0.273295652667362</v>
+        <v>0.32069923129363798</v>
       </c>
       <c r="F10" s="1">
-        <v>0.283869583869583</v>
+        <v>0.23754262574595</v>
       </c>
       <c r="G10" s="1">
-        <v>0.59090909090909005</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.24285714285714199</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -3168,22 +3173,22 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>4440</v>
       </c>
       <c r="D11" s="1">
-        <v>0.40559748005628798</v>
+        <v>0.43006070211936898</v>
       </c>
       <c r="E11" s="1">
-        <v>0.37376555556616903</v>
+        <v>0.35143182926090399</v>
       </c>
       <c r="F11" s="1">
-        <v>0.54805194805194801</v>
+        <v>0.50714285714285701</v>
       </c>
       <c r="G11" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -3191,22 +3196,22 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>4412</v>
       </c>
       <c r="D12" s="1">
-        <v>0.34167744685178603</v>
+        <v>0.31448894920065001</v>
       </c>
       <c r="E12" s="1">
-        <v>0.482392249134174</v>
+        <v>0.36523914130991503</v>
       </c>
       <c r="F12" s="1">
-        <v>0.25</v>
+        <v>0.206349206349206</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -3214,16 +3219,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>4443</v>
       </c>
       <c r="D13" s="1">
-        <v>0.61264340099625303</v>
+        <v>0.63824030318217395</v>
       </c>
       <c r="E13" s="1">
-        <v>0.755298342892046</v>
+        <v>0.725319079069079</v>
       </c>
       <c r="F13" s="1">
-        <v>0.79166666666666596</v>
+        <v>0.80555555555555503</v>
       </c>
       <c r="G13" s="1">
         <v>0</v>
@@ -3237,9 +3242,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82367681-20B8-422B-BAF8-1E957EF58DE1}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3260,7 +3265,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -3268,22 +3273,22 @@
         <v>2014</v>
       </c>
       <c r="C2" s="1">
-        <v>4921</v>
+        <v>4229</v>
       </c>
       <c r="D2" s="1">
-        <v>0.79049894152815503</v>
+        <v>0.81592307961400601</v>
       </c>
       <c r="E2" s="1">
-        <v>0.60057846422314998</v>
+        <v>0.610180689252383</v>
       </c>
       <c r="F2" s="1">
-        <v>0.50888931321227604</v>
+        <v>0.51045631893599297</v>
       </c>
       <c r="G2" s="1">
-        <v>0.49600149681275901</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.498895705939854</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -3291,22 +3296,22 @@
         <v>2015</v>
       </c>
       <c r="C3" s="1">
-        <v>5014</v>
+        <v>4294</v>
       </c>
       <c r="D3" s="1">
-        <v>0.81841518232205401</v>
+        <v>0.85691277906977903</v>
       </c>
       <c r="E3" s="1">
-        <v>0.56453423261997204</v>
+        <v>0.57494245566839997</v>
       </c>
       <c r="F3" s="1">
-        <v>0.50331052756414696</v>
+        <v>0.50508452783186797</v>
       </c>
       <c r="G3" s="1">
-        <v>0.49600605193270503</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.50022692233880295</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -3314,22 +3319,22 @@
         <v>2016</v>
       </c>
       <c r="C4" s="1">
-        <v>4829</v>
+        <v>4199</v>
       </c>
       <c r="D4" s="1">
-        <v>0.83158120049566397</v>
+        <v>0.82987016339147601</v>
       </c>
       <c r="E4" s="1">
-        <v>0.58307301731297001</v>
+        <v>0.58950290766361302</v>
       </c>
       <c r="F4" s="1">
-        <v>0.51119417748454199</v>
+        <v>0.51293371714879799</v>
       </c>
       <c r="G4" s="1">
-        <v>0.49280763772352798</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.48650193079496901</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -3337,22 +3342,22 @@
         <v>2017</v>
       </c>
       <c r="C5" s="1">
-        <v>4946</v>
+        <v>4257</v>
       </c>
       <c r="D5" s="1">
-        <v>0.81171748897565699</v>
+        <v>0.85015143643501401</v>
       </c>
       <c r="E5" s="1">
-        <v>0.58182078887185795</v>
+        <v>0.59535237703639998</v>
       </c>
       <c r="F5" s="1">
-        <v>0.51071964053636099</v>
+        <v>0.51528003773666398</v>
       </c>
       <c r="G5" s="1">
-        <v>0.50050768732778494</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.50341944546800499</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -3360,22 +3365,22 @@
         <v>2018</v>
       </c>
       <c r="C6" s="1">
-        <v>4943</v>
+        <v>4235</v>
       </c>
       <c r="D6" s="1">
-        <v>0.86016727534499804</v>
+        <v>0.92139117688482397</v>
       </c>
       <c r="E6" s="1">
-        <v>0.55555153521553102</v>
+        <v>0.56502813692017395</v>
       </c>
       <c r="F6" s="1">
-        <v>0.50554495696261503</v>
+        <v>0.506445537749874</v>
       </c>
       <c r="G6" s="1">
-        <v>0.50019235883871804</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.50056763536523596</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -3383,22 +3388,22 @@
         <v>2019</v>
       </c>
       <c r="C7" s="1">
-        <v>4841</v>
+        <v>4179</v>
       </c>
       <c r="D7" s="1">
-        <v>0.88820971737938204</v>
+        <v>0.95692747615356299</v>
       </c>
       <c r="E7" s="1">
-        <v>0.56637881773697296</v>
+        <v>0.57723659444750297</v>
       </c>
       <c r="F7" s="1">
-        <v>0.45460672127141</v>
+        <v>0.43015626907974602</v>
       </c>
       <c r="G7" s="1">
-        <v>0.15971069115011899</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.15892767127378199</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -3406,22 +3411,22 @@
         <v>2020</v>
       </c>
       <c r="C8" s="1">
-        <v>4855</v>
+        <v>4197</v>
       </c>
       <c r="D8" s="1">
-        <v>0.81147693421240696</v>
+        <v>0.86827400303178703</v>
       </c>
       <c r="E8" s="1">
-        <v>0.56098613482114401</v>
+        <v>0.57095627519185599</v>
       </c>
       <c r="F8" s="1">
-        <v>0.50481341260208601</v>
+        <v>0.50557896369775401</v>
       </c>
       <c r="G8" s="1">
-        <v>0.49742029097373303</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.49952095352985798</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -3429,22 +3434,22 @@
         <v>2021</v>
       </c>
       <c r="C9" s="1">
-        <v>5131</v>
+        <v>4260</v>
       </c>
       <c r="D9" s="1">
-        <v>0.84697517925340504</v>
+        <v>0.89189799634223299</v>
       </c>
       <c r="E9" s="1">
-        <v>0.57856852274371995</v>
+        <v>0.58856248571440795</v>
       </c>
       <c r="F9" s="1">
-        <v>0.50536469930253003</v>
+        <v>0.50646051459615504</v>
       </c>
       <c r="G9" s="1">
-        <v>0.50019482709466201</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.50023441050650397</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -3452,22 +3457,22 @@
         <v>2022</v>
       </c>
       <c r="C10" s="1">
-        <v>5129</v>
+        <v>4414</v>
       </c>
       <c r="D10" s="1">
-        <v>0.667579534616911</v>
+        <v>0.68598287740987496</v>
       </c>
       <c r="E10" s="1">
-        <v>0.54439160805687103</v>
+        <v>0.54728425986484996</v>
       </c>
       <c r="F10" s="1">
-        <v>0.50279910239472903</v>
+        <v>0.50191526052423996</v>
       </c>
       <c r="G10" s="1">
-        <v>0.49830956417099198</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.499168744553244</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -3475,22 +3480,22 @@
         <v>2023</v>
       </c>
       <c r="C11" s="1">
-        <v>5161</v>
+        <v>4440</v>
       </c>
       <c r="D11" s="1">
-        <v>0.629276097612253</v>
+        <v>0.65056294596574205</v>
       </c>
       <c r="E11" s="1">
-        <v>0.52298193803325099</v>
+        <v>0.52683402605892604</v>
       </c>
       <c r="F11" s="1">
-        <v>0.50107537927051504</v>
+        <v>0.50124829153505002</v>
       </c>
       <c r="G11" s="1">
-        <v>0.16637591166462501</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>0.16771790497276101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -3498,22 +3503,22 @@
         <v>2024</v>
       </c>
       <c r="C12" s="1">
-        <v>5122</v>
+        <v>4412</v>
       </c>
       <c r="D12" s="1">
-        <v>0.57364013806553604</v>
+        <v>0.58521316615470997</v>
       </c>
       <c r="E12" s="1">
-        <v>0.51063263807566805</v>
+        <v>0.51107853785048696</v>
       </c>
       <c r="F12" s="1">
-        <v>0.49960760031489199</v>
+        <v>0.49988232577117803</v>
       </c>
       <c r="G12" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -3521,16 +3526,16 @@
         <v>2025</v>
       </c>
       <c r="C13" s="1">
-        <v>5114</v>
+        <v>4443</v>
       </c>
       <c r="D13" s="1">
-        <v>0.56370258449509103</v>
+        <v>0.573412241668661</v>
       </c>
       <c r="E13" s="1">
-        <v>0.51285093577989604</v>
+        <v>0.51479537015963395</v>
       </c>
       <c r="F13" s="1">
-        <v>0.50048897834968697</v>
+        <v>0.50056272063726404</v>
       </c>
       <c r="G13" s="1">
         <v>0</v>

</xml_diff>